<commit_message>
Add DOI column to publications spreadsheet
New add_doi_column.py fills in DOIs by title match without disturbing
manual edits already made to the spreadsheet. fetch_openalex.py also
includes DOI now so future full regenerations have it too.
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -2,28 +2,41 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Publications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -53,13 +66,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -422,14 +438,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,6 +475,11 @@
           <t>Co-authors</t>
         </is>
       </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>DOI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -483,6 +505,11 @@
           <t>Catherine M Sniezek, Christopher D. McGann, Rashmi Karki, Ross Giglio, Benjamin A. Garcia, Jose L McFaline-Figueroa, Devin K. Schweppe</t>
         </is>
       </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s42003-025-09455-0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -508,6 +535,11 @@
           <t>Cameron S. Movassaghi, Jie Sun, Yuming Jiang, Natalie Turner, Vincent Chang, Nara Chung, Ryan Chen, Elizabeth N. Browne, Devin K. Schweppe, Stacy A. Malaker, Jesse G. Meyer</t>
         </is>
       </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acs.analchem.4c06750</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -533,6 +565,11 @@
           <t>Sayan Kundu, Rajendra Rohokale, Sixue Chen, Shayak Biswas, Zhongwu Guo</t>
         </is>
       </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jlr.2024.100570</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -558,6 +595,11 @@
           <t>Natasha I. Edman, Ashish Phal, Rachel L. Redler, Thomas Schlichthaerle, Sanjay Srivatsan, Devon Duron Ehnes, Ali Etemadi, Seong Jin An, Andrew Favor, Zhe Li, Florian Praetorius, Max Gordon, Thomas L. Vincent, Silvia Marchianò, Leslie P. Blakely, Wei Yang, Brian Coventry, Derrick R. Hicks, Longxing Cao, Neville P. Bethel, Piper Heine, Analisa Murray, Stacey Gerben, Lauren Carter, Marcos C. Miranda, Babak Negahdari, Sangwon Lee, Cole Trapnell, Ying Zheng, Charles E. Murry, Devin K. Schweppe, Benjamin Freedman, Lance Stewart, Damian C. Ekiert, Joseph Schlessinger, Jay Shendure, Gira Bhabha, Hannele Ruohola‐Baker, David Baker</t>
         </is>
       </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.cell.2024.05.025</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -583,6 +625,11 @@
           <t>Zachary T. Baumer, Luke Erber, Elizabeth A. Jolley, Sheldon Lawrence, Shino Murakami, Veronica C. Perez, Wil Prall, Cassandra Schaening-Burgos, Megan M. Sylvia, Sixue Chen, Brian D. Gregory</t>
         </is>
       </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.tibs.2023.09.011</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -608,6 +655,11 @@
           <t>Dawei Dai, Guimei Zhao, Sarah Joe, Sixue Chen</t>
         </is>
       </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jprot.2023.104903</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -633,6 +685,11 @@
           <t>Sayan Kundu, Mohit Jaiswal, Venkannababu Mullapudi, Kendall C. Craig, Sixue Chen, Zhongwu Guo</t>
         </is>
       </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acs.jproteome.2c00728</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -658,6 +715,11 @@
           <t>Chris D McGann, William D. Barshop, Jesse D. Canterbury, Wassim Gabriel, Jingjing Huang, David Bergen, Vlad Zabrouskov, Rafael D. Melani, Mathias Wilhelm, Graeme C. McAlister, Devin K. Schweppe</t>
         </is>
       </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acs.jproteome.3c00085</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -673,14 +735,19 @@
           <t>International Journal of Molecular Sciences</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>article</t>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>review</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Ramesh Katam, Kirstie Grant, Chaquayla S. Katam, Sixue Chen</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ijms23136985</t>
         </is>
       </c>
     </row>
@@ -693,9 +760,9 @@
       <c r="B11" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Methods in enzymology on CD-ROM/Methods in enzymology</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Methods in enzymology</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -706,6 +773,11 @@
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>In-Cheol Yeo, Craig Dufresne, Guimei Zhao, Sarah Joe, Sixue Chen</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/bs.mie.2022.06.005</t>
         </is>
       </c>
     </row>
@@ -733,11 +805,16 @@
           <t>Aneirin A. Lott, Wei Zhu, Craig Dufresne, Sixue Chen</t>
         </is>
       </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ijms23020880</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Effect of Sonication on Plant Stomatal Movement</t>
+          <t>Proteomics and phosphoproteomics revealed molecular networks of stomatal immune responses</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -745,7 +822,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>UF Journal of Undergraduate Research</t>
+          <t>Planta</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -755,14 +832,19 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Suren Jeevaratnam, Sixue Chen</t>
+          <t>Qiuying Pang, Tong Zhang, Aiqin Zhang, Wenwen Kong, Sixue Chen</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s00425-020-03474-3</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Proteomics and phosphoproteomics revealed molecular networks of stomatal immune responses</t>
+          <t>Proteomics data of SNF1-related protein kinase 2.4 interacting proteins revealed by immunoprecipitation-mass spectrometry</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -770,92 +852,82 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Planta</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+          <t>Data in Brief</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>article</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Qiuying Pang, Tong Zhang, Aiqin Zhang, Wenwen Kong, Sixue Chen</t>
+          <t>Tong Zhang, Jacqueline D. Schneider, Jin Koh, Sixue Chen</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.dib.2020.106326</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Proteomics data of SNF1-related protein kinase 2.4 interacting proteins revealed by immunoprecipitation-mass spectrometry</t>
+          <t>MPK4 Phosphorylation Dynamics and Interacting Proteins in Plant Immunity</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Data in Brief</t>
+          <t>Journal of Proteome Research</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>data-paper</t>
+          <t>article</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Tong Zhang, Jacqueline D. Schneider, Jin Koh, Sixue Chen</t>
+          <t>Tong Zhang, Jacqueline D. Schneider, Sisi Geng, Tianyi Ma, Sheldon Lawrence, Craig Dufresne, Alice Harmon, Sixue Chen</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acs.jproteome.8b00345</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>MPK4 Phosphorylation Dynamics and Interacting Proteins in Plant Immunity</t>
+          <t>New functions of an old kinase MPK4 in guard cells</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Journal of Proteome Research</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>article</t>
+          <t>Plant Signaling &amp; Behavior</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>review</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Tong Zhang, Jacqueline D. Schneider, Sisi Geng, Tianyi Ma, Sheldon Lawrence, Craig Dufresne, Alice Harmon, Sixue Chen</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>New functions of an old kinase MPK4 in guard cells</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Plant Signaling &amp; Behavior</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
           <t>Sixun Chen</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/15592324.2018.1477908</t>
         </is>
       </c>
     </row>

</xml_diff>